<commit_message>
feat : data tabungan umum, karyawan, dinamis
</commit_message>
<xml_diff>
--- a/public/assets/files/Contoh Import Sikas - Data Tabungan Karyawan.xlsx
+++ b/public/assets/files/Contoh Import Sikas - Data Tabungan Karyawan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wazirul\Documents\Sikas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30800434-3D31-40B0-85D3-6C3895E6D667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F8AF29-C4F6-43C3-AD3C-7AF8E7F4F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,66 +46,42 @@
     <t>Total Tabungan</t>
   </si>
   <si>
-    <t>NIP</t>
-  </si>
-  <si>
     <t>Jabatan</t>
   </si>
   <si>
-    <t>003219340</t>
-  </si>
-  <si>
     <t>Buhanuddin</t>
   </si>
   <si>
     <t>Guru</t>
   </si>
   <si>
-    <t>003122341</t>
-  </si>
-  <si>
     <t>Loehoet Suparjo</t>
   </si>
   <si>
     <t>Kepala Sekolah</t>
   </si>
   <si>
-    <t>001242313</t>
-  </si>
-  <si>
     <t>Sri Puan</t>
   </si>
   <si>
     <t>Ketua Komite</t>
   </si>
   <si>
-    <t>005315543</t>
-  </si>
-  <si>
     <t>Wiwik Sutini</t>
   </si>
   <si>
     <t>Bendahara Komite</t>
   </si>
   <si>
-    <t>009324123</t>
-  </si>
-  <si>
     <t>Sunaryadi</t>
   </si>
   <si>
     <t>Manager AVM</t>
   </si>
   <si>
-    <t>003412312</t>
-  </si>
-  <si>
     <t>Harto Djatmoko</t>
   </si>
   <si>
-    <t>009931251</t>
-  </si>
-  <si>
     <t>Fahmi Jaelani</t>
   </si>
   <si>
@@ -119,6 +95,30 @@
   </si>
   <si>
     <t>1. Pastikan Jabatan Karyawan yang akan di import sudah dibuat oleh Admin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO BUKU TABUNGAN </t>
+  </si>
+  <si>
+    <t>0001</t>
+  </si>
+  <si>
+    <t>0002</t>
+  </si>
+  <si>
+    <t>0003</t>
+  </si>
+  <si>
+    <t>0004</t>
+  </si>
+  <si>
+    <t>0005</t>
+  </si>
+  <si>
+    <t>0006</t>
+  </si>
+  <si>
+    <t>0007</t>
   </si>
 </sst>
 </file>
@@ -128,7 +128,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-[$Rp-421]* #,##0_-;\-[$Rp-421]* #,##0_-;_-[$Rp-421]* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -139,6 +139,25 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -146,20 +165,28 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="4">
@@ -206,36 +233,49 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{460DE5C9-1B66-4F2A-AFF2-AFEE35D99331}"/>
+    <cellStyle name="Normal 3" xfId="3" xr:uid="{F537AC0F-F128-472F-A0F6-93FE92FDC8B9}"/>
+    <cellStyle name="Normal 4" xfId="1" xr:uid="{98ABB563-45FA-42FE-891E-712088581D80}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -457,7 +497,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.33203125" customWidth="1"/>
     <col min="2" max="2" width="22.109375" customWidth="1"/>
@@ -466,156 +506,157 @@
     <col min="7" max="7" width="67.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" ht="30" customHeight="1">
+      <c r="A1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="F1" s="6"/>
+      <c r="G1" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="13.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="4">
+      <c r="E2" s="2">
         <v>500000</v>
       </c>
-      <c r="G2" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="G2" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="13.2">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="B3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="2">
         <v>50000</v>
       </c>
-      <c r="G3" s="8"/>
-    </row>
-    <row r="4" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:7" ht="13.2">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="4">
+      <c r="B4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2">
         <v>250000</v>
       </c>
-      <c r="G4" s="8"/>
-    </row>
-    <row r="5" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:7" ht="13.2">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="4">
+      <c r="B5" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2">
         <v>380000</v>
       </c>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" spans="1:7" ht="13.2">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="2">
+        <v>75000</v>
+      </c>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2">
+        <v>380000</v>
+      </c>
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="4">
+      <c r="B8" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2">
         <v>75000</v>
       </c>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="4">
-        <v>380000</v>
-      </c>
-      <c r="G7" s="8"/>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="4">
-        <v>75000</v>
-      </c>
-      <c r="G8" s="8"/>
+      <c r="G8" s="5"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>